<commit_message>
Enrich product sample data to a believable quarter
Signing Log now seeds 16 signings across Jan-Mar (3 companies, varied appt
types and statuses), with matching Mileage Log (14 drives, 343 mi) and
Expenses (9 rows across deductible categories). The Dashboard charts and
Tax Summary now populate meaningfully on first open.
Verified: fees $1,385 · outstanding $230 · net $1,154.40 · deduction $240.10.
</commit_message>
<xml_diff>
--- a/dist/Signing-Agent-HQ.xlsx
+++ b/dist/Signing-Agent-HQ.xlsx
@@ -2139,17 +2139,51 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="10" t="n"/>
-      <c r="I10" s="13" t="n"/>
-      <c r="J10" s="10" t="n"/>
-      <c r="K10" s="9" t="n"/>
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Coastal Signings</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>CS-1063</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>D. Nguyen</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Refi</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>160</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>160</v>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I10" s="13" t="n">
+        <v>38</v>
+      </c>
+      <c r="J10" s="10" t="n">
+        <v>125</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="L10" s="9">
         <f>IF(G10="","",G10-(I10*Settings!$B$4)-(J10*0.1)-K10)</f>
         <v/>
@@ -2160,17 +2194,51 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="9" t="n"/>
-      <c r="H11" s="10" t="n"/>
-      <c r="I11" s="13" t="n"/>
-      <c r="J11" s="10" t="n"/>
-      <c r="K11" s="9" t="n"/>
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>BlueRock Escrow</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>BR-219</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>A. Silva</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Purchase</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="L11" s="9">
         <f>IF(G11="","",G11-(I11*Settings!$B$4)-(J11*0.1)-K11)</f>
         <v/>
@@ -2181,17 +2249,51 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="10" t="n"/>
-      <c r="I12" s="13" t="n"/>
-      <c r="J12" s="10" t="n"/>
-      <c r="K12" s="9" t="n"/>
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Summit Title</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>ST-1041</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>L. Romano</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>HELOC</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I12" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="J12" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="L12" s="9">
         <f>IF(G12="","",G12-(I12*Settings!$B$4)-(J12*0.1)-K12)</f>
         <v/>
@@ -2202,17 +2304,51 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="10" t="n"/>
-      <c r="I13" s="13" t="n"/>
-      <c r="J13" s="10" t="n"/>
-      <c r="K13" s="9" t="n"/>
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Coastal Signings</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>CS-1079</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>G. Patel</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Apostille</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I13" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="J13" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="L13" s="9">
         <f>IF(G13="","",G13-(I13*Settings!$B$4)-(J13*0.1)-K13)</f>
         <v/>
@@ -2223,17 +2359,51 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="10" t="n"/>
-      <c r="I14" s="13" t="n"/>
-      <c r="J14" s="10" t="n"/>
-      <c r="K14" s="9" t="n"/>
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>BlueRock Escrow</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>BR-233</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>H. Kim</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Refi</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>105</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>105</v>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I14" s="13" t="n">
+        <v>44</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>115</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="L14" s="9">
         <f>IF(G14="","",G14-(I14*Settings!$B$4)-(J14*0.1)-K14)</f>
         <v/>
@@ -2244,17 +2414,51 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="9" t="n"/>
-      <c r="H15" s="10" t="n"/>
-      <c r="I15" s="13" t="n"/>
-      <c r="J15" s="10" t="n"/>
-      <c r="K15" s="9" t="n"/>
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Summit Title</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>ST-1067</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>N. Brooks</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>RON</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="L15" s="9">
         <f>IF(G15="","",G15-(I15*Settings!$B$4)-(J15*0.1)-K15)</f>
         <v/>
@@ -2265,17 +2469,51 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="9" t="n"/>
-      <c r="G16" s="9" t="n"/>
-      <c r="H16" s="10" t="n"/>
-      <c r="I16" s="13" t="n"/>
-      <c r="J16" s="10" t="n"/>
-      <c r="K16" s="9" t="n"/>
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Coastal Signings</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>CS-1090</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>P. Adams</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Purchase</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>165</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>165</v>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="n">
+        <v>28</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>130</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <v>5</v>
+      </c>
       <c r="L16" s="9">
         <f>IF(G16="","",G16-(I16*Settings!$B$4)-(J16*0.1)-K16)</f>
         <v/>
@@ -2286,17 +2524,51 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="9" t="n"/>
-      <c r="G17" s="9" t="n"/>
-      <c r="H17" s="10" t="n"/>
-      <c r="I17" s="13" t="n"/>
-      <c r="J17" s="10" t="n"/>
-      <c r="K17" s="9" t="n"/>
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>BlueRock Escrow</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>BR-248</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>S. Lopez</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Invoiced</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>85</v>
+      </c>
+      <c r="K17" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="L17" s="9">
         <f>IF(G17="","",G17-(I17*Settings!$B$4)-(J17*0.1)-K17)</f>
         <v/>
@@ -2307,17 +2579,51 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="9" t="n"/>
-      <c r="G18" s="9" t="n"/>
-      <c r="H18" s="10" t="n"/>
-      <c r="I18" s="13" t="n"/>
-      <c r="J18" s="10" t="n"/>
-      <c r="K18" s="9" t="n"/>
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Summit Title</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>ST-1090</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>J. Wu</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Refi</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="n">
+        <v>33</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>120</v>
+      </c>
+      <c r="K18" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="L18" s="9">
         <f>IF(G18="","",G18-(I18*Settings!$B$4)-(J18*0.1)-K18)</f>
         <v/>
@@ -2328,17 +2634,51 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="9" t="n"/>
-      <c r="G19" s="9" t="n"/>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="13" t="n"/>
-      <c r="J19" s="10" t="n"/>
-      <c r="K19" s="9" t="n"/>
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Coastal Signings</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>CS-1108</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>R. Diaz</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>HELOC</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>145</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>145</v>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I19" s="13" t="n">
+        <v>22</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="K19" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="L19" s="9">
         <f>IF(G19="","",G19-(I19*Settings!$B$4)-(J19*0.1)-K19)</f>
         <v/>
@@ -2349,17 +2689,51 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="9" t="n"/>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="10" t="n"/>
-      <c r="I20" s="13" t="n"/>
-      <c r="J20" s="10" t="n"/>
-      <c r="K20" s="9" t="n"/>
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>BlueRock Escrow</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>BR-260</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>T. Evans</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Refi</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>Cancelled</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="L20" s="9">
         <f>IF(G20="","",G20-(I20*Settings!$B$4)-(J20*0.1)-K20)</f>
         <v/>
@@ -8483,132 +8857,348 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n"/>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="13" t="n"/>
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>BR-204 signing</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Lakewood</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>32</v>
+      </c>
       <c r="F7" s="9">
         <f>IF(E7="","",E7*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="13" t="n"/>
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>CS-1051 signing</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Midtown</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>12</v>
+      </c>
       <c r="F8" s="9">
         <f>IF(E8="","",E8*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="13" t="n"/>
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>ST-1007 signing</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Eastside</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>27</v>
+      </c>
       <c r="F9" s="9">
         <f>IF(E9="","",E9*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="13" t="n"/>
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>CS-1063 signing</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Hillcrest</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>38</v>
+      </c>
       <c r="F10" s="9">
         <f>IF(E10="","",E10*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="13" t="n"/>
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>BR-219 signing</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Parkview</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>21</v>
+      </c>
       <c r="F11" s="9">
         <f>IF(E11="","",E11*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="13" t="n"/>
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>ST-1041 signing</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Northgate</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>16</v>
+      </c>
       <c r="F12" s="9">
         <f>IF(E12="","",E12*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="13" t="n"/>
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>CS-1079 apostille</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>City Hall</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>9</v>
+      </c>
       <c r="F13" s="9">
         <f>IF(E13="","",E13*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="13" t="n"/>
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>BR-233 signing</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Westend</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>44</v>
+      </c>
       <c r="F14" s="9">
         <f>IF(E14="","",E14*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="13" t="n"/>
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>CS-1090 signing</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Bayfront</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>28</v>
+      </c>
       <c r="F15" s="9">
         <f>IF(E15="","",E15*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="13" t="n"/>
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>BR-248 signing</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Southside</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>19</v>
+      </c>
       <c r="F16" s="9">
         <f>IF(E16="","",E16*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="13" t="n"/>
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>ST-1090 signing</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Uptown</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>33</v>
+      </c>
       <c r="F17" s="9">
         <f>IF(E17="","",E17*Settings!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="13" t="n"/>
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>CS-1108 signing</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Riverside</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>22</v>
+      </c>
       <c r="F18" s="9">
         <f>IF(E18="","",E18*Settings!$B$4)</f>
         <v/>
@@ -11377,39 +11967,129 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="10" t="n"/>
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>NNA Membership</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>NNA</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="10" t="n"/>
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Local FB ads</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="10" t="n"/>
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Training/Education</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>LSS course</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="10" t="n"/>
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Phone/Internet</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Carrier (biz %)</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="10" t="n"/>
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Toner + paper</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="n"/>

</xml_diff>